<commit_message>
Update MNT-Halan (HALN) valuation model
Version HALN preview link to bust Office viewer cache.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/MNT-HALN-Valuation-Model.xlsx
+++ b/models/MNT-HALN-Valuation-Model.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Valuations\HALN - CA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6EAA8F-B806-4DB1-8850-971A56C1D749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB07D556-316C-41C5-B6E9-173468F884A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="646" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1010,7 +1010,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-EGP 10-year government bond yield: Cbonds index 23.35% on 12 Oct 2026. Confirm against the latest Ministry of Finance 10-year auction before publishing.</t>
+EGP 10-year government bond yield: Cbonds index 23.35% on 12 Oct 2026.</t>
         </r>
       </text>
     </comment>
@@ -1058,65 +1058,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-5.0% = middle of a 4.5-5.5% mature-market (US implied) premium. Egypt country risk is already inside the EGP 10-year yield in C6, so Damodaran's total Egypt premium (13.94%) would count it twice. Update from Damodaran's latest monthly implied ERP and write the date here.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Ahmed Wael:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-"Industry" uses C23 as published; "Blume-adjusted" pulls it toward 1. HALN has no trading history yet (listing expected 20 Oct 2026), so there is no observed beta. Once peer or HALN betas exist, regress 104 weekly returns on the EGX30.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Ahmed Wael</author>
-  </authors>
-  <commentList>
-    <comment ref="D36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Ahmed Wael:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Book multiples on the two lenders only (Contact Financial, CI Capital). Fawry and e-finance are asset-light payment platforms; their P/B (8-10x) says nothing about a balance-sheet lender.</t>
+5.0% = middle of a 4.5-5.5% mature-market (US implied) premium. Egypt country risk is already inside the EGP 10-year yield in C6, so Damodaran's total Egypt premium (13.94%) would count it twice.</t>
         </r>
       </text>
     </comment>
@@ -2225,18 +2167,6 @@
     <t>PEER STATISTICS</t>
   </si>
   <si>
-    <t>P/E (all)</t>
-  </si>
-  <si>
-    <t>P/B (lenders)</t>
-  </si>
-  <si>
-    <t>P/TBV (lenders)</t>
-  </si>
-  <si>
-    <t>ROE (all)</t>
-  </si>
-  <si>
     <t>Mean</t>
   </si>
   <si>
@@ -2298,6 +2228,18 @@
   </si>
   <si>
     <t>USD/EGP</t>
+  </si>
+  <si>
+    <t>P/B</t>
+  </si>
+  <si>
+    <t>P/TBV</t>
+  </si>
+  <si>
+    <t>ROE</t>
+  </si>
+  <si>
+    <t>P/E</t>
   </si>
 </sst>
 </file>
@@ -14526,7 +14468,7 @@
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B32" s="284" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="C32" s="285">
         <f>D8</f>
@@ -14759,7 +14701,7 @@
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B50" s="201" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="C50" s="288">
         <f ca="1">C49/C51</f>
@@ -14775,7 +14717,7 @@
     </row>
     <row r="51" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="201" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="C51" s="127">
         <v>50</v>
@@ -15222,7 +15164,7 @@
       <formula>#REF!="Industry"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" sqref="C21" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Industry,Blume-adjusted"</formula1>
     </dataValidation>
@@ -15234,7 +15176,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B1:I70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -15758,16 +15700,16 @@
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.25">
       <c r="C36" s="44" t="s">
-        <v>366</v>
+        <v>390</v>
       </c>
       <c r="D36" s="44" t="s">
-        <v>367</v>
+        <v>387</v>
       </c>
       <c r="E36" s="44" t="s">
-        <v>368</v>
+        <v>388</v>
       </c>
       <c r="F36" s="44" t="s">
-        <v>369</v>
+        <v>389</v>
       </c>
       <c r="G36" s="44"/>
     </row>
@@ -15780,19 +15722,19 @@
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B38" s="35" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="C38" s="149">
         <f>AVERAGE(C30:F30)</f>
         <v>19.345791137266943</v>
       </c>
       <c r="D38" s="149">
-        <f>AVERAGE(E31:F31)</f>
-        <v>1.2477779033630894</v>
+        <f>AVERAGE(C31:F31)</f>
+        <v>5.1052706414588993</v>
       </c>
       <c r="E38" s="149">
-        <f>AVERAGE(E32:F32)</f>
-        <v>1.304441547496455</v>
+        <f>AVERAGE(C32:F32)</f>
+        <v>5.7107200931403943</v>
       </c>
       <c r="F38" s="1">
         <f>AVERAGE(C33:F33)</f>
@@ -15802,19 +15744,19 @@
     </row>
     <row r="39" spans="2:7" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B39" s="44" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="C39" s="150">
         <f>MEDIAN(C30:F30)</f>
         <v>17.822519791535356</v>
       </c>
       <c r="D39" s="150">
-        <f>MEDIAN(E31:F31)</f>
-        <v>1.2477779033630894</v>
+        <f>MEDIAN(C31:F31)</f>
+        <v>4.8370113736834313</v>
       </c>
       <c r="E39" s="150">
-        <f>MEDIAN(E32:F32)</f>
-        <v>1.304441547496455</v>
+        <f>MEDIAN(C32:F32)</f>
+        <v>5.6980566128732537</v>
       </c>
       <c r="F39" s="167">
         <f>MEDIAN(C33:F33)</f>
@@ -15824,19 +15766,19 @@
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B40" s="35" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="C40" s="149">
         <f>MAX(C30:F30)</f>
         <v>34.732926313227686</v>
       </c>
       <c r="D40" s="149">
-        <f>MAX(E31:F31)</f>
-        <v>1.4337199699095724</v>
+        <f>MAX(C31:F31)</f>
+        <v>9.6852239816521308</v>
       </c>
       <c r="E40" s="149">
-        <f>MAX(E32:F32)</f>
-        <v>1.5196377063320523</v>
+        <f>MAX(C32:F32)</f>
+        <v>10.357521758154215</v>
       </c>
       <c r="F40" s="1">
         <f>MAX(C33:F33)</f>
@@ -15846,18 +15788,18 @@
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B41" s="35" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C41" s="149">
         <f>MIN(C30:F30)</f>
         <v>7.0051986527693701</v>
       </c>
       <c r="D41" s="149">
-        <f>MIN(E31:F31)</f>
+        <f>MIN(C31:F31)</f>
         <v>1.0618358368166061</v>
       </c>
       <c r="E41" s="149">
-        <f>MIN(E32:F32)</f>
+        <f>MIN(C32:F32)</f>
         <v>1.089245388660858</v>
       </c>
       <c r="F41" s="1">
@@ -15868,7 +15810,7 @@
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B43" s="145" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="C43" s="146"/>
       <c r="D43" s="146"/>
@@ -15878,12 +15820,12 @@
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B44" s="44" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B45" s="35" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C45" s="149">
         <f>C39</f>
@@ -15892,7 +15834,7 @@
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B46" s="35" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="C46" s="151">
         <f>$G$23</f>
@@ -15901,7 +15843,7 @@
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B47" s="35" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C47" s="151">
         <f>C45*C46</f>
@@ -15919,7 +15861,7 @@
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49" s="44" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C49" s="249">
         <f>C47/C48</f>
@@ -15928,21 +15870,21 @@
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51" s="44" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52" s="35" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="C52" s="149">
         <f>D39</f>
-        <v>1.2477779033630894</v>
+        <v>4.8370113736834313</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53" s="35" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="C53" s="151">
         <f>G24</f>
@@ -15951,11 +15893,11 @@
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54" s="35" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C54" s="151">
         <f>C52*C53</f>
-        <v>11374432050.214367</v>
+        <v>44092988862.671463</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.25">
@@ -15969,11 +15911,11 @@
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56" s="44" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C56" s="249">
         <f>C54/C55</f>
-        <v>7.1090200313839791</v>
+        <v>27.558118039169663</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.25">
@@ -15982,21 +15924,21 @@
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58" s="44" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59" s="35" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="C59" s="149">
         <f>E39</f>
-        <v>1.304441547496455</v>
+        <v>5.6980566128732537</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60" s="35" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="C60" s="151">
         <f>G27</f>
@@ -16005,11 +15947,11 @@
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61" s="35" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C61" s="151">
         <f>C59*C60</f>
-        <v>11186259613.377829</v>
+        <v>48863776752.325317</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.25">
@@ -16023,21 +15965,21 @@
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63" s="44" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C63" s="249">
         <f>C61/C62</f>
-        <v>6.9914122583611427</v>
+        <v>30.539860470203323</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65" s="44" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66" s="35" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="C66" s="149">
         <f>MEDIAN(E30:F30)</f>
@@ -16046,7 +15988,7 @@
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67" s="35" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="C67" s="151">
         <f>G23</f>
@@ -16055,7 +15997,7 @@
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68" s="35" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C68" s="151">
         <f>C66*C67</f>
@@ -16073,7 +16015,7 @@
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70" s="44" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C70" s="249">
         <f>C68/C69</f>
@@ -16082,7 +16024,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>